<commit_message>
Remaining calibration file updates
</commit_message>
<xml_diff>
--- a/InputData/trans/TTS/Transportation Technology Shareweights.xlsx
+++ b/InputData/trans/TTS/Transportation Technology Shareweights.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\TTS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\EPS Structure Research\eps-us-calibration\InputData\trans\TTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06641E14-21DC-4145-949A-E72A3CBD9CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00CB3D61-2644-4B08-8BA5-549C12CAEB60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="10008" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="89">
   <si>
     <t>TTS Transportation Technology Shareweights</t>
   </si>
@@ -275,6 +275,45 @@
   </si>
   <si>
     <t>Max Fraction of Production (dimensionless)</t>
+  </si>
+  <si>
+    <t>Calibration record (2026-09-22)</t>
+  </si>
+  <si>
+    <t>On-road anchors (Data tab columns D-E) rewritten by calibration/steps/03-trans-shareweights/solve_base_year.py:</t>
+  </si>
+  <si>
+    <t>logit inversion at the start year from 'BAU New Vehicle Cost per Mile' in the BAU export and observed technology shares</t>
+  </si>
+  <si>
+    <t>(calibration/benchmarks/vehicle-technology-shares.csv), ZEV-mandate correction for passenger LDVs (3 passes), then the</t>
+  </si>
+  <si>
+    <t>existing s-curve formulas carry the trajectory to the unchanged 2050 targets. Confirmed by a headless run after the third pass.</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-psgr natural gas vehicle: IT-year cell set to =E11 (was an s-curve formula)</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-psgr gasoline vehicle: IT-year cell set to =E12 (was an s-curve formula)</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-psgr diesel vehicle: IT-year cell set to =E13 (was an s-curve formula)</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-psgr plugin hybrid vehicle: 2050 target pinned at its pre-calibration value 0.091009</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-psgr LPG vehicle: IT-year cell set to =E15 (was an s-curve formula)</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-psgr hydrogen vehicle: IT-year cell set to =E16 (was an s-curve formula)</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-frgt battery electric vehicle: IT-year cell set to =E17 (was an s-curve formula)</t>
+  </si>
+  <si>
+    <t>TTS-LDVs-frgt plugin hybrid vehicle: 2050 target pinned at its pre-calibration value 0.00100885</t>
   </si>
 </sst>
 </file>
@@ -1044,18 +1083,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B53"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B67"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="63.42578125" customWidth="1"/>
+    <col min="2" max="2" width="63.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1063,193 +1102,258 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B39" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B44" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B47" s="1"/>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B53" s="1"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>88</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1266,12 +1370,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -1384,7 +1488,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -1497,7 +1601,7 @@
         <v>0.93664816810144857</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1610,7 +1714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -1723,7 +1827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1836,7 +1940,7 @@
         <v>6.3351831898551425E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -1949,7 +2053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -2062,7 +2166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -2186,12 +2290,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -2304,7 +2408,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -2417,7 +2521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -2530,7 +2634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -2643,7 +2747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -2756,7 +2860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -2869,7 +2973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -2982,7 +3086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -3106,12 +3210,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -3224,7 +3328,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -3337,7 +3441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -3450,7 +3554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -3563,7 +3667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -3676,7 +3780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -3789,7 +3893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -3902,7 +4006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -4026,12 +4130,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -4144,7 +4248,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -4257,7 +4361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -4370,7 +4474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -4483,7 +4587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -4596,7 +4700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -4709,7 +4813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -4822,7 +4926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -4946,12 +5050,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -5064,233 +5168,233 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
       <c r="B2">
         <f>Data!I80</f>
-        <v>0.18123793393000001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="C2">
         <f>Data!J80</f>
-        <v>0.23279812904258823</v>
+        <v>0.20439829056518796</v>
       </c>
       <c r="D2">
         <f>Data!K80</f>
-        <v>0.24933658275197695</v>
+        <v>0.22154895526074969</v>
       </c>
       <c r="E2">
         <f>Data!L80</f>
-        <v>0.2705622726537894</v>
+        <v>0.24356036556758487</v>
       </c>
       <c r="F2">
         <f>Data!M80</f>
-        <v>0.29738020490215311</v>
+        <v>0.27137102863815177</v>
       </c>
       <c r="G2">
         <f>Data!N80</f>
-        <v>0.33060103270559432</v>
+        <v>0.30582160597612668</v>
       </c>
       <c r="H2">
         <f>Data!O80</f>
-        <v>0.37076106043634494</v>
+        <v>0.34746825456114855</v>
       </c>
       <c r="I2">
         <f>Data!P80</f>
-        <v>0.41790151635931294</v>
+        <v>0.39635372882237035</v>
       </c>
       <c r="J2">
         <f>Data!Q80</f>
-        <v>0.47136110874344317</v>
+        <v>0.45179225771102483</v>
       </c>
       <c r="K2">
         <f>Data!R80</f>
-        <v>0.52966825809683538</v>
+        <v>0.5122577876502824</v>
       </c>
       <c r="L2">
         <f>Data!S80</f>
-        <v>0.59061896696500005</v>
+        <v>0.57546473487299998</v>
       </c>
       <c r="M2">
         <f>Data!T80</f>
-        <v>0.65156967583316472</v>
+        <v>0.63867168209571767</v>
       </c>
       <c r="N2">
         <f>Data!U80</f>
-        <v>0.70987682518655681</v>
+        <v>0.69913721203497514</v>
       </c>
       <c r="O2">
         <f>Data!V80</f>
-        <v>0.76333641757068704</v>
+        <v>0.75457574092362967</v>
       </c>
       <c r="P2">
         <f>Data!W80</f>
-        <v>0.81047687349365505</v>
+        <v>0.80346121518485136</v>
       </c>
       <c r="Q2">
         <f>Data!X80</f>
-        <v>0.85063690122440572</v>
+        <v>0.84510786376987324</v>
       </c>
       <c r="R2">
         <f>Data!Y80</f>
-        <v>0.88385772902784698</v>
+        <v>0.87955844110784831</v>
       </c>
       <c r="S2">
         <f>Data!Z80</f>
-        <v>0.91067566127621058</v>
+        <v>0.9073691041784151</v>
       </c>
       <c r="T2">
         <f>Data!AA80</f>
-        <v>0.93190135117802309</v>
+        <v>0.92938051448525039</v>
       </c>
       <c r="U2">
         <f>Data!AB80</f>
-        <v>0.94843980488741186</v>
+        <v>0.94653117918081209</v>
       </c>
       <c r="V2">
         <f>Data!AC80</f>
-        <v>0.96116949409196173</v>
+        <v>0.95973208871336446</v>
       </c>
       <c r="W2">
         <f>Data!AD80</f>
-        <v>0.97087565957856936</v>
+        <v>0.96979755146251745</v>
       </c>
       <c r="X2">
         <f>Data!AE80</f>
-        <v>0.97822339058775476</v>
+        <v>0.97741727656052824</v>
       </c>
       <c r="Y2">
         <f>Data!AF80</f>
-        <v>0.98375551028570629</v>
+        <v>0.98315418108996533</v>
       </c>
       <c r="Z2">
         <f>Data!AG80</f>
-        <v>0.98790358328663208</v>
+        <v>0.98745580507620323</v>
       </c>
       <c r="AA2">
         <f>Data!AH80</f>
-        <v>0.99100430815198304</v>
+        <v>0.990671310794772</v>
       </c>
       <c r="AB2">
         <f>Data!AI80</f>
-        <v>0.99331679637819548</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+        <v>0.99306940138275057</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
       <c r="B3">
         <f>Data!I81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="C3">
         <f>Data!J81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="D3">
         <f>Data!K81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="E3">
         <f>Data!L81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="F3">
         <f>Data!M81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="G3">
         <f>Data!N81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="H3">
         <f>Data!O81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="I3">
         <f>Data!P81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="J3">
         <f>Data!Q81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="K3">
         <f>Data!R81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="L3">
         <f>Data!S81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="M3">
         <f>Data!T81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="N3">
         <f>Data!U81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="O3">
         <f>Data!V81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="P3">
         <f>Data!W81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Q3">
         <f>Data!X81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="R3">
         <f>Data!Y81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="S3">
         <f>Data!Z81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="T3">
         <f>Data!AA81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="U3">
         <f>Data!AB81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="V3">
         <f>Data!AC81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="W3">
         <f>Data!AD81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="X3">
         <f>Data!AE81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Y3">
         <f>Data!AF81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Z3">
         <f>Data!AG81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AA3">
         <f>Data!AH81</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AB3">
         <f>Data!AI81</f>
-        <v>1.06732008758E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+        <v>1.0695408416000001E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -5403,233 +5507,233 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
       <c r="B5">
         <f>Data!I83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="C5">
         <f>Data!J83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="D5">
         <f>Data!K83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="E5">
         <f>Data!L83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="F5">
         <f>Data!M83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="G5">
         <f>Data!N83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="H5">
         <f>Data!O83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="I5">
         <f>Data!P83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="J5">
         <f>Data!Q83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="K5">
         <f>Data!R83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="L5">
         <f>Data!S83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="M5">
         <f>Data!T83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="N5">
         <f>Data!U83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="O5">
         <f>Data!V83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="P5">
         <f>Data!W83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Q5">
         <f>Data!X83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="R5">
         <f>Data!Y83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="S5">
         <f>Data!Z83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="T5">
         <f>Data!AA83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="U5">
         <f>Data!AB83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="V5">
         <f>Data!AC83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="W5">
         <f>Data!AD83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="X5">
         <f>Data!AE83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Y5">
         <f>Data!AF83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Z5">
         <f>Data!AG83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AA5">
         <f>Data!AH83</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AB5">
         <f>Data!AI83</f>
-        <v>6.7938858436000005E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+        <v>6.7938939010499994E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
       <c r="B6">
         <f>Data!I84</f>
-        <v>1.3970074369600001E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="C6">
         <f>Data!J84</f>
-        <v>1.5110140554321749E-2</v>
+        <v>1.2806537318706219E-2</v>
       </c>
       <c r="D6">
         <f>Data!K84</f>
-        <v>1.550108920235292E-2</v>
+        <v>1.3208673429906077E-2</v>
       </c>
       <c r="E6">
         <f>Data!L84</f>
-        <v>1.6022481838446352E-2</v>
+        <v>1.3744986339907847E-2</v>
       </c>
       <c r="F6">
         <f>Data!M84</f>
-        <v>1.6714992675043627E-2</v>
+        <v>1.4457314202391682E-2</v>
       </c>
       <c r="G6">
         <f>Data!N84</f>
-        <v>1.7629781849127387E-2</v>
+        <v>1.5398281162851517E-2</v>
       </c>
       <c r="H6">
         <f>Data!O84</f>
-        <v>1.8829532862010948E-2</v>
+        <v>1.663236448596514E-2</v>
       </c>
       <c r="I6">
         <f>Data!P84</f>
-        <v>2.0388253288765361E-2</v>
+        <v>1.8235689562083129E-2</v>
       </c>
       <c r="J6">
         <f>Data!Q84</f>
-        <v>2.2388737554300295E-2</v>
+        <v>2.0293420077612576E-2</v>
       </c>
       <c r="K6">
         <f>Data!R84</f>
-        <v>2.4916280910733307E-2</v>
+        <v>2.2893292110330199E-2</v>
       </c>
       <c r="L6">
         <f>Data!S84</f>
-        <v>2.8047286009566623E-2</v>
+        <v>2.611389466499453E-2</v>
       </c>
       <c r="M6">
         <f>Data!T84</f>
-        <v>3.18322986028182E-2</v>
+        <v>3.0007219920774212E-2</v>
       </c>
       <c r="N6">
         <f>Data!U84</f>
-        <v>3.6275204382572757E-2</v>
+        <v>3.4577264763480553E-2</v>
       </c>
       <c r="O6">
         <f>Data!V84</f>
-        <v>4.1313677756162917E-2</v>
+        <v>3.9759920079065703E-2</v>
       </c>
       <c r="P6">
         <f>Data!W84</f>
-        <v>4.6809024922225891E-2</v>
+        <v>4.5412523177152192E-2</v>
       </c>
       <c r="Q6">
         <f>Data!X84</f>
-        <v>5.2553522963420404E-2</v>
+        <v>5.1321406900666118E-2</v>
       </c>
       <c r="R6">
         <f>Data!Y84</f>
-        <v>5.8298021004614918E-2</v>
+        <v>5.7230290624180044E-2</v>
       </c>
       <c r="S6">
         <f>Data!Z84</f>
-        <v>6.3793368170677878E-2</v>
+        <v>6.2882893722266534E-2</v>
       </c>
       <c r="T6">
         <f>Data!AA84</f>
-        <v>6.8831841544268038E-2</v>
+        <v>6.8065549037851683E-2</v>
       </c>
       <c r="U6">
         <f>Data!AB84</f>
-        <v>7.3274747324022602E-2</v>
+        <v>7.2635593880558014E-2</v>
       </c>
       <c r="V6">
         <f>Data!AC84</f>
-        <v>7.7059759917274179E-2</v>
+        <v>7.6528919136337692E-2</v>
       </c>
       <c r="W6">
         <f>Data!AD84</f>
-        <v>8.0190765016107501E-2</v>
+        <v>7.9749521691002051E-2</v>
       </c>
       <c r="X6">
         <f>Data!AE84</f>
-        <v>8.2718308372540517E-2</v>
+        <v>8.234939372371966E-2</v>
       </c>
       <c r="Y6">
         <f>Data!AF84</f>
-        <v>8.4718792638075455E-2</v>
+        <v>8.4407124239249121E-2</v>
       </c>
       <c r="Z6">
         <f>Data!AG84</f>
-        <v>8.6277513064829864E-2</v>
+        <v>8.601044931536711E-2</v>
       </c>
       <c r="AA6">
         <f>Data!AH84</f>
-        <v>8.7477264077713432E-2</v>
+        <v>8.7244532638480726E-2</v>
       </c>
       <c r="AB6">
         <f>Data!AI84</f>
-        <v>8.8392053251797179E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+        <v>8.8185499598940564E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -5742,7 +5846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -5866,12 +5970,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -5984,7 +6088,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -6070,7 +6174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -6156,7 +6260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -6242,7 +6346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -6328,7 +6432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -6414,7 +6518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -6500,7 +6604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -6594,18 +6698,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="8" width="23.28515625" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="24.5546875" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="8" width="23.33203125" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -6631,7 +6735,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -6658,7 +6762,7 @@
       </c>
       <c r="J2" s="3"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -6686,7 +6790,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="18"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -6712,7 +6816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -6738,7 +6842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>48</v>
       </c>
@@ -6764,7 +6868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -6790,7 +6894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -6810,20 +6914,20 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:AK93"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="24.109375" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" customWidth="1"/>
     <col min="6" max="6" width="18" style="5" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" customWidth="1"/>
-    <col min="8" max="9" width="9.140625" customWidth="1"/>
-    <col min="14" max="14" width="11.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" customWidth="1"/>
+    <col min="8" max="9" width="9.109375" customWidth="1"/>
+    <col min="14" max="14" width="11.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>50</v>
       </c>
@@ -6852,7 +6956,7 @@
       </c>
       <c r="X1" s="11"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -6887,7 +6991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -6925,7 +7029,7 @@
         <v>-0.3</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:37" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -6963,12 +7067,12 @@
         <v>-14</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -6986,7 +7090,7 @@
       <c r="O6" s="16"/>
       <c r="R6" s="19"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9" t="s">
@@ -7002,7 +7106,7 @@
       <c r="G7" s="2"/>
       <c r="N7" s="19"/>
     </row>
-    <row r="8" spans="1:37" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -7015,7 +7119,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>68</v>
       </c>
@@ -7145,7 +7249,7 @@
       <c r="AJ9" s="15"/>
       <c r="AK9" s="15"/>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>44</v>
       </c>
@@ -7156,10 +7260,10 @@
         <v>37</v>
       </c>
       <c r="D10">
-        <v>0.18218700570900001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="E10" s="16">
-        <v>0.18123793393000001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -7170,126 +7274,126 @@
       </c>
       <c r="I10">
         <f>D10</f>
-        <v>0.18218700570900001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="J10" s="16">
         <f>E10</f>
-        <v>0.18123793393000001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="K10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:K$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,K$9))</f>
-        <v>0.22006843983803839</v>
+        <v>0.19119738103263559</v>
       </c>
       <c r="L10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:L$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,L$9))</f>
-        <v>0.23279812904258823</v>
+        <v>0.20439829056518796</v>
       </c>
       <c r="M10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:M$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,M$9))</f>
-        <v>0.24933658275197695</v>
+        <v>0.22154895526074969</v>
       </c>
       <c r="N10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:N$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,N$9))</f>
-        <v>0.2705622726537894</v>
+        <v>0.24356036556758487</v>
       </c>
       <c r="O10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:O$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,O$9))</f>
-        <v>0.29738020490215311</v>
+        <v>0.27137102863815177</v>
       </c>
       <c r="P10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:P$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,P$9))</f>
-        <v>0.33060103270559432</v>
+        <v>0.30582160597612668</v>
       </c>
       <c r="Q10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:Q$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,Q$9))</f>
-        <v>0.37076106043634494</v>
+        <v>0.34746825456114855</v>
       </c>
       <c r="R10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:R$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,R$9))</f>
-        <v>0.41790151635931294</v>
+        <v>0.39635372882237035</v>
       </c>
       <c r="S10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:S$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,S$9))</f>
-        <v>0.47136110874344317</v>
+        <v>0.45179225771102483</v>
       </c>
       <c r="T10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:T$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,T$9))</f>
-        <v>0.52966825809683538</v>
+        <v>0.5122577876502824</v>
       </c>
       <c r="U10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:U$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,U$9))</f>
-        <v>0.59061896696500005</v>
+        <v>0.57546473487299998</v>
       </c>
       <c r="V10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:V$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,V$9))</f>
-        <v>0.65156967583316472</v>
+        <v>0.63867168209571767</v>
       </c>
       <c r="W10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:W$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,W$9))</f>
-        <v>0.70987682518655681</v>
+        <v>0.69913721203497514</v>
       </c>
       <c r="X10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:X$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,X$9))</f>
-        <v>0.76333641757068704</v>
+        <v>0.75457574092362967</v>
       </c>
       <c r="Y10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:Y$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,Y$9))</f>
-        <v>0.81047687349365505</v>
+        <v>0.80346121518485136</v>
       </c>
       <c r="Z10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:Z$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,Z$9))</f>
-        <v>0.85063690122440572</v>
+        <v>0.84510786376987324</v>
       </c>
       <c r="AA10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AA$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AA$9))</f>
-        <v>0.88385772902784698</v>
+        <v>0.87955844110784831</v>
       </c>
       <c r="AB10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AB$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AB$9))</f>
-        <v>0.91067566127621058</v>
+        <v>0.9073691041784151</v>
       </c>
       <c r="AC10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AC$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AC$9))</f>
-        <v>0.93190135117802309</v>
+        <v>0.92938051448525039</v>
       </c>
       <c r="AD10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AD$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AD$9))</f>
-        <v>0.94843980488741186</v>
+        <v>0.94653117918081209</v>
       </c>
       <c r="AE10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AE$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AE$9))</f>
-        <v>0.96116949409196173</v>
+        <v>0.95973208871336446</v>
       </c>
       <c r="AF10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AF$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AF$9))</f>
-        <v>0.97087565957856936</v>
+        <v>0.96979755146251745</v>
       </c>
       <c r="AG10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AG$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AG$9))</f>
-        <v>0.97822339058775476</v>
+        <v>0.97741727656052824</v>
       </c>
       <c r="AH10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AH$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AH$9))</f>
-        <v>0.98375551028570629</v>
+        <v>0.98315418108996533</v>
       </c>
       <c r="AI10">
         <f>IF($G10="s-curve",$E10+($F10-$E10)*$O$2/(1+EXP($O$3*(COUNT($K$9:AI$9)+$O$4))),TREND($E10:$F10,$E$9:$F$9,AI$9))</f>
-        <v>0.98790358328663208</v>
-      </c>
-    </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+        <v>0.98745580507620323</v>
+      </c>
+    </row>
+    <row r="11" spans="1:37" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>38</v>
       </c>
       <c r="D11">
-        <v>1.06995776452E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="E11" s="16">
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="F11" s="16">
         <f>E11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="G11" s="5" t="str">
         <f>IF(E11=F11,"n/a",IF(OR(C11="battery electric vehicle",C11="natural gas vehicle",C11="plugin hybrid vehicle"),"s-curve","linear"))</f>
@@ -7297,114 +7401,114 @@
       </c>
       <c r="I11" s="16">
         <f>E11</f>
-        <v>1.06732008758E-4</v>
-      </c>
-      <c r="J11">
-        <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,J$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
+      </c>
+      <c r="J11" s="16">
+        <f>E11</f>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="K11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,K$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="L11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,L$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="M11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,M$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="N11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,N$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="O11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,O$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="P11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,P$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Q11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,Q$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="R11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,R$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="S11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,S$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="T11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,T$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="U11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,U$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="V11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,V$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="W11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,W$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="X11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,X$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Y11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,Y$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Z11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,Z$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AA11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AA$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AB11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AB$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AC11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AC$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AD11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AD$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AE11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AE$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AF11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AF$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AG11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AG$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AH11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AH$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AI11">
         <f>IF($G11="s-curve",$E11+($F11-$E11)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E11:$F11,$E$9:$F$9,AI$9))</f>
-        <v>1.06732008758E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+        <v>1.0695408416000001E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:37" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
         <v>39</v>
       </c>
@@ -7426,7 +7530,7 @@
         <v>1</v>
       </c>
       <c r="J12">
-        <f>IF($G12="s-curve",$E12+($F12-$E12)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E12:$F12,$E$9:$F$9,J$9))</f>
+        <f>E12</f>
         <v>1</v>
       </c>
       <c r="K12">
@@ -7530,19 +7634,19 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>40</v>
       </c>
       <c r="D13">
-        <v>6.8106756297200005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="E13" s="16">
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="F13" s="16">
         <f>E13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="G13" s="5" t="str">
         <f>IF(E13=F13,"n/a",IF(OR(C13="battery electric vehicle",C13="natural gas vehicle",C13="plugin hybrid vehicle"),"s-curve","linear"))</f>
@@ -7550,126 +7654,125 @@
       </c>
       <c r="I13" s="16">
         <f>E13</f>
-        <v>6.7938858436000005E-2</v>
-      </c>
-      <c r="J13">
-        <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,J$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
+      </c>
+      <c r="J13" s="16">
+        <f>E13</f>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="K13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,K$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="L13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,L$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="M13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,M$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="N13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,N$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="O13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,O$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="P13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,P$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Q13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,Q$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="R13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,R$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="S13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,S$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="T13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,T$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="U13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,U$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="V13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,V$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="W13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,W$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="X13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,X$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Y13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,Y$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Z13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,Z$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AA13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AA$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AB13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AB$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AC13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AC$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AD13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AD$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AE13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AE$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AF13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AF$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AG13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AG$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AH13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AH$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AI13">
         <f>IF($G13="s-curve",$E13+($F13-$E13)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E13:$F13,$E$9:$F$9,AI$9))</f>
-        <v>6.7938858436000005E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+        <v>6.7938939010499994E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:37" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
         <v>41</v>
       </c>
       <c r="D14">
-        <v>1.6603971957400002E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="E14" s="16">
-        <v>1.3970074369600001E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="F14" s="23">
-        <f>D14/D10*F10</f>
-        <v>9.1136971557240806E-2</v>
+        <v>9.1008967024832244E-2</v>
       </c>
       <c r="G14" s="5" t="str">
         <f>IF(E14=F14,"n/a",IF(OR(C14="battery electric vehicle",C14="natural gas vehicle",C14="plugin hybrid vehicle",C14="hydrogen vehicle"),"s-curve","linear"))</f>
@@ -7677,114 +7780,114 @@
       </c>
       <c r="I14">
         <f>D14</f>
-        <v>1.6603971957400002E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="J14">
         <f>E14</f>
-        <v>1.3970074369600001E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="K14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:K$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,K$9))</f>
-        <v>1.6992371673937554E-2</v>
+        <v>1.4742630733106016E-2</v>
       </c>
       <c r="L14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:L$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,L$9))</f>
-        <v>1.8393603157554242E-2</v>
+        <v>1.6183960131609255E-2</v>
       </c>
       <c r="M14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:M$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,M$9))</f>
-        <v>2.0388253288765361E-2</v>
+        <v>1.8235689562083126E-2</v>
       </c>
       <c r="N14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:N$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,N$9))</f>
-        <v>2.3168593997747108E-2</v>
+        <v>2.109559304595815E-2</v>
       </c>
       <c r="O14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:O$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,O$9))</f>
-        <v>2.6932694373384324E-2</v>
+        <v>2.4967407656003776E-2</v>
       </c>
       <c r="P14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:P$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,P$9))</f>
-        <v>3.18322986028182E-2</v>
+        <v>3.0007219920774209E-2</v>
       </c>
       <c r="Q14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:Q$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,Q$9))</f>
-        <v>3.7893781709970521E-2</v>
+        <v>3.6242159617047354E-2</v>
       </c>
       <c r="R14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:R$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,R$9))</f>
-        <v>4.493810244183398E-2</v>
+        <v>4.3488062012213696E-2</v>
       </c>
       <c r="S14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:S$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,S$9))</f>
-        <v>5.2553522963420404E-2</v>
+        <v>5.1321406900666118E-2</v>
       </c>
       <c r="T14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:T$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,T$9))</f>
-        <v>6.0168943485006829E-2</v>
+        <v>5.9154751789118533E-2</v>
       </c>
       <c r="U14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:U$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,U$9))</f>
-        <v>6.721326421687028E-2</v>
+        <v>6.6400654184284882E-2</v>
       </c>
       <c r="V14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:V$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,V$9))</f>
-        <v>7.3274747324022602E-2</v>
+        <v>7.2635593880558028E-2</v>
       </c>
       <c r="W14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:W$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,W$9))</f>
-        <v>7.8174351553456478E-2</v>
+        <v>7.7675406145328446E-2</v>
       </c>
       <c r="X14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:X$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,X$9))</f>
-        <v>8.1938451929093686E-2</v>
+        <v>8.1547220755374072E-2</v>
       </c>
       <c r="Y14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:Y$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,Y$9))</f>
-        <v>8.4718792638075455E-2</v>
+        <v>8.4407124239249121E-2</v>
       </c>
       <c r="Z14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:Z$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,Z$9))</f>
-        <v>8.6713442769286567E-2</v>
+        <v>8.6458853669722974E-2</v>
       </c>
       <c r="AA14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AA$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AA$9))</f>
-        <v>8.8114674252903258E-2</v>
+        <v>8.7900183068226223E-2</v>
       </c>
       <c r="AB14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AB$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AB$9))</f>
-        <v>8.908456408839445E-2</v>
+        <v>8.8897827461424384E-2</v>
       </c>
       <c r="AC14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AC$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AC$9))</f>
-        <v>8.9749031542300767E-2</v>
+        <v>8.9581309446279456E-2</v>
       </c>
       <c r="AD14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AD$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AD$9))</f>
-        <v>9.0201057861762329E-2</v>
+        <v>9.0046271039531389E-2</v>
       </c>
       <c r="AE14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AE$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AE$9))</f>
-        <v>9.050709126827812E-2</v>
+        <v>9.0361061958014605E-2</v>
       </c>
       <c r="AF14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AF$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AF$9))</f>
-        <v>9.0713610894126245E-2</v>
+        <v>9.0573491389970062E-2</v>
       </c>
       <c r="AG14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AG$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AG$9))</f>
-        <v>9.0852670195706434E-2</v>
+        <v>9.0716530039790799E-2</v>
       </c>
       <c r="AH14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AH$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AH$9))</f>
-        <v>9.0946166900329001E-2</v>
+        <v>9.0812702264445544E-2</v>
       </c>
       <c r="AI14">
         <f>IF($G14="s-curve",$E14+($F14-$E14)*$U$2/(1+EXP($U$3*(COUNT($I$9:AI$9)+$U$4))),TREND($E14:$F14,$E$9:$F$9,AI$9))</f>
-        <v>9.1008967024832244E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+        <v>9.0877299489625335E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:37" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
         <v>42</v>
       </c>
@@ -7806,8 +7909,8 @@
         <f>E15</f>
         <v>0</v>
       </c>
-      <c r="J15">
-        <f>IF($G15="s-curve",$E15+($F15-$E15)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E15:$F15,$E$9:$F$9,J$9))</f>
+      <c r="J15" s="16">
+        <f>E15</f>
         <v>0</v>
       </c>
       <c r="K15">
@@ -7911,7 +8014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:37" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:37" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="17"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17" t="s">
@@ -7935,8 +8038,8 @@
         <f>E16</f>
         <v>0</v>
       </c>
-      <c r="J16">
-        <f>IF($G16="s-curve",$E16+($F16-$E16)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E16:$F16,$E$9:$F$9,J$9))</f>
+      <c r="J16" s="16">
+        <f>E16</f>
         <v>0</v>
       </c>
       <c r="K16">
@@ -8040,7 +8143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>44</v>
       </c>
@@ -8068,8 +8171,8 @@
         <v>0.30732944248799998</v>
       </c>
       <c r="J17">
-        <f>IF($G17="s-curve",$E17+($F17-$E17)*$X$2/(1+EXP($X$3*(COUNT($I$9:J$9)+$X$4))),TREND($E17:$F17,$E$9:$F$9,J$9))</f>
-        <v>0.30713450135322462</v>
+        <f>E17</f>
+        <v>0.30732944248799998</v>
       </c>
       <c r="K17" s="25">
         <f>IF($G17="s-curve",$D17+($F17-$D17)*$X$2/(1+EXP($X$3*(COUNT($I$9:K$9)+$X$4))),TREND($D17:$F17,$E$9:$F$9,K$9))</f>
@@ -8172,7 +8275,7 @@
         <v>0.30014541837982223</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
         <v>38</v>
       </c>
@@ -8298,7 +8401,7 @@
         <v>0.59353215226599998</v>
       </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
         <v>39</v>
       </c>
@@ -8425,7 +8528,7 @@
         <v>0.97401567340499995</v>
       </c>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
         <v>40</v>
       </c>
@@ -8551,7 +8654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
         <v>41</v>
       </c>
@@ -8562,8 +8665,7 @@
         <v>1.03300009982E-3</v>
       </c>
       <c r="F21" s="16">
-        <f>E21/E17*F17</f>
-        <v>1.0083642733256849E-3</v>
+        <v>1.0088530556553437E-3</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>74</v>
@@ -8578,106 +8680,106 @@
       </c>
       <c r="K21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:K$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,K$9))</f>
-        <v>1.0321237741728829E-3</v>
+        <v>1.0321411607416443E-3</v>
       </c>
       <c r="L21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:L$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,L$9))</f>
-        <v>1.0318317242370562E-3</v>
+        <v>1.0318549051658338E-3</v>
       </c>
       <c r="M21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:M$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,M$9))</f>
-        <v>1.0314486991464152E-3</v>
+        <v>1.031479479410095E-3</v>
       </c>
       <c r="N21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:N$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,N$9))</f>
-        <v>1.0309510717001113E-3</v>
+        <v>1.0309917250444676E-3</v>
       </c>
       <c r="O21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:O$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,O$9))</f>
-        <v>1.0303124094619435E-3</v>
+        <v>1.030365734060366E-3</v>
       </c>
       <c r="P21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:P$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,P$9))</f>
-        <v>1.0295054815970778E-3</v>
+        <v>1.0295748158910443E-3</v>
       </c>
       <c r="Q21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:Q$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,Q$9))</f>
-        <v>1.028505896267372E-3</v>
+        <v>1.0285950626398874E-3</v>
       </c>
       <c r="R21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:R$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,R$9))</f>
-        <v>1.0272975165485478E-3</v>
+        <v>1.0274106575441273E-3</v>
       </c>
       <c r="S21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:S$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,S$9))</f>
-        <v>1.025879101918574E-3</v>
+        <v>1.0260203846940701E-3</v>
       </c>
       <c r="T21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:T$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,T$9))</f>
-        <v>1.024270550060824E-3</v>
+        <v>1.0244437469969668E-3</v>
       </c>
       <c r="U21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:U$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,U$9))</f>
-        <v>1.0225161395008146E-3</v>
+        <v>1.0227241444788512E-3</v>
       </c>
       <c r="V21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:V$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,V$9))</f>
-        <v>1.0206821865728424E-3</v>
+        <v>1.0209265777376718E-3</v>
       </c>
       <c r="W21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:W$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,W$9))</f>
-        <v>1.0188482336448703E-3</v>
+        <v>1.0191290109964925E-3</v>
       </c>
       <c r="X21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:X$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,X$9))</f>
-        <v>1.0170938230848608E-3</v>
+        <v>1.0174094084783769E-3</v>
       </c>
       <c r="Y21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:Y$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,Y$9))</f>
-        <v>1.0154852712271109E-3</v>
+        <v>1.0158327707812736E-3</v>
       </c>
       <c r="Z21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:Z$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,Z$9))</f>
-        <v>1.0140668565971371E-3</v>
+        <v>1.0144424979312164E-3</v>
       </c>
       <c r="AA21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AA$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AA$9))</f>
-        <v>1.0128584768783128E-3</v>
+        <v>1.0132580928354563E-3</v>
       </c>
       <c r="AB21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AB$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AB$9))</f>
-        <v>1.0118588915486071E-3</v>
+        <v>1.0122783395842994E-3</v>
       </c>
       <c r="AC21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AC$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AC$9))</f>
-        <v>1.0110519636837413E-3</v>
+        <v>1.0114874214149777E-3</v>
       </c>
       <c r="AD21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AD$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AD$9))</f>
-        <v>1.0104133014455735E-3</v>
+        <v>1.0108614304308761E-3</v>
       </c>
       <c r="AE21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AE$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AE$9))</f>
-        <v>1.0099156739992697E-3</v>
+        <v>1.0103736760652487E-3</v>
       </c>
       <c r="AF21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AF$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AF$9))</f>
-        <v>1.0095326489086287E-3</v>
+        <v>1.0099982503095099E-3</v>
       </c>
       <c r="AG21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AG$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AG$9))</f>
-        <v>1.0092405989728019E-3</v>
+        <v>1.0097119947336994E-3</v>
       </c>
       <c r="AH21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AH$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AH$9))</f>
-        <v>1.0090195122447148E-3</v>
+        <v>1.0094952944338913E-3</v>
       </c>
       <c r="AI21">
         <f>IF($G21="s-curve",$E21+($F21-$E21)*$X$2/(1+EXP($X$3*(COUNT($I$9:AI$9)+$X$4))),TREND($E21:$F21,$E$9:$F$9,AI$9))</f>
-        <v>1.0088530556553437E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
+        <v>1.0093321403941448E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C22" t="s">
         <v>42</v>
       </c>
@@ -8804,7 +8906,7 @@
         <v>1.3472785756799999E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="17"/>
       <c r="B23" s="17"/>
       <c r="C23" s="17" t="s">
@@ -8933,7 +9035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>45</v>
       </c>
@@ -9065,7 +9167,7 @@
         <v>0.73751575888521737</v>
       </c>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C25" t="s">
         <v>38</v>
       </c>
@@ -9192,7 +9294,7 @@
         <v>1.5317430015500001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C26" t="s">
         <v>39</v>
       </c>
@@ -9319,7 +9421,7 @@
         <v>0.38138758163300002</v>
       </c>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C27" t="s">
         <v>40</v>
       </c>
@@ -9445,7 +9547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C28" t="s">
         <v>41</v>
       </c>
@@ -9572,7 +9674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C29" t="s">
         <v>42</v>
       </c>
@@ -9699,7 +9801,7 @@
         <v>5.5226931821800003E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="17"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17" t="s">
@@ -9828,7 +9930,7 @@
         <v>2.0026390066599999E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>45</v>
       </c>
@@ -9960,7 +10062,7 @@
         <v>0.24513810124032956</v>
       </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C32" t="s">
         <v>38</v>
       </c>
@@ -10087,7 +10189,7 @@
         <v>2.32516282526E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C33" t="s">
         <v>39</v>
       </c>
@@ -10214,7 +10316,7 @@
         <v>7.3518745439599999E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C34" t="s">
         <v>40</v>
       </c>
@@ -10340,7 +10442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C35" t="s">
         <v>41</v>
       </c>
@@ -10467,7 +10569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C36" t="s">
         <v>42</v>
       </c>
@@ -10594,7 +10696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="17"/>
       <c r="B37" s="17"/>
       <c r="C37" s="17" t="s">
@@ -10723,7 +10825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>46</v>
       </c>
@@ -10852,7 +10954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C39" t="s">
         <v>38</v>
       </c>
@@ -10975,7 +11077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C40" t="s">
         <v>39</v>
       </c>
@@ -11098,7 +11200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C41" t="s">
         <v>40</v>
       </c>
@@ -11221,7 +11323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C42" t="s">
         <v>41</v>
       </c>
@@ -11344,7 +11446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C43" t="s">
         <v>42</v>
       </c>
@@ -11467,7 +11569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="17"/>
       <c r="B44" s="17"/>
       <c r="C44" s="17" t="s">
@@ -11593,7 +11695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -11722,7 +11824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C46" t="s">
         <v>38</v>
       </c>
@@ -11845,7 +11947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C47" t="s">
         <v>39</v>
       </c>
@@ -11968,7 +12070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C48" t="s">
         <v>40</v>
       </c>
@@ -12091,7 +12193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C49" t="s">
         <v>41</v>
       </c>
@@ -12214,7 +12316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C50" t="s">
         <v>42</v>
       </c>
@@ -12337,7 +12439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="17"/>
       <c r="B51" s="17"/>
       <c r="C51" s="17" t="s">
@@ -12463,7 +12565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>47</v>
       </c>
@@ -12593,7 +12695,7 @@
         <v>0.93664816810144857</v>
       </c>
     </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C53" t="s">
         <v>38</v>
       </c>
@@ -12716,7 +12818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C54" t="s">
         <v>39</v>
       </c>
@@ -12839,7 +12941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C55" t="s">
         <v>40</v>
       </c>
@@ -12964,7 +13066,7 @@
         <v>6.3351831898551425E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C56" t="s">
         <v>41</v>
       </c>
@@ -13087,7 +13189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C57" t="s">
         <v>42</v>
       </c>
@@ -13210,7 +13312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="17"/>
       <c r="B58" s="17"/>
       <c r="C58" s="17" t="s">
@@ -13336,7 +13438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>47</v>
       </c>
@@ -13465,7 +13567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C60" t="s">
         <v>38</v>
       </c>
@@ -13588,7 +13690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C61" t="s">
         <v>39</v>
       </c>
@@ -13711,7 +13813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C62" t="s">
         <v>40</v>
       </c>
@@ -13834,7 +13936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C63" t="s">
         <v>41</v>
       </c>
@@ -13957,7 +14059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C64" t="s">
         <v>42</v>
       </c>
@@ -14080,7 +14182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="17"/>
       <c r="B65" s="17"/>
       <c r="C65" s="17" t="s">
@@ -14206,7 +14308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>48</v>
       </c>
@@ -14335,7 +14437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C67" t="s">
         <v>38</v>
       </c>
@@ -14458,7 +14560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C68" t="s">
         <v>39</v>
       </c>
@@ -14581,7 +14683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C69" t="s">
         <v>40</v>
       </c>
@@ -14704,7 +14806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C70" t="s">
         <v>41</v>
       </c>
@@ -14827,7 +14929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C71" t="s">
         <v>42</v>
       </c>
@@ -14950,7 +15052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A72" s="17"/>
       <c r="B72" s="17"/>
       <c r="C72" s="17" t="s">
@@ -15076,7 +15178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>48</v>
       </c>
@@ -15205,7 +15307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C74" t="s">
         <v>38</v>
       </c>
@@ -15328,7 +15430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C75" t="s">
         <v>39</v>
       </c>
@@ -15451,7 +15553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C76" t="s">
         <v>40</v>
       </c>
@@ -15574,7 +15676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C77" t="s">
         <v>41</v>
       </c>
@@ -15697,7 +15799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C78" t="s">
         <v>42</v>
       </c>
@@ -15820,7 +15922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A79" s="17"/>
       <c r="B79" s="17"/>
       <c r="C79" s="17" t="s">
@@ -15946,7 +16048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>49</v>
       </c>
@@ -15958,11 +16060,11 @@
       </c>
       <c r="D80">
         <f t="shared" ref="D80:F86" si="5">D10</f>
-        <v>0.18218700570900001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="E80">
         <f t="shared" si="5"/>
-        <v>0.18123793393000001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="F80">
         <f t="shared" si="5"/>
@@ -15974,128 +16076,128 @@
       </c>
       <c r="I80" s="16">
         <f t="shared" si="4"/>
-        <v>0.18123793393000001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="J80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:J$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,J$9))</f>
-        <v>0.23279812904258823</v>
+        <v>0.20439829056518796</v>
       </c>
       <c r="K80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:K$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,K$9))</f>
-        <v>0.24933658275197695</v>
+        <v>0.22154895526074969</v>
       </c>
       <c r="L80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:L$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,L$9))</f>
-        <v>0.2705622726537894</v>
+        <v>0.24356036556758487</v>
       </c>
       <c r="M80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:M$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,M$9))</f>
-        <v>0.29738020490215311</v>
+        <v>0.27137102863815177</v>
       </c>
       <c r="N80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:N$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,N$9))</f>
-        <v>0.33060103270559432</v>
+        <v>0.30582160597612668</v>
       </c>
       <c r="O80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:O$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,O$9))</f>
-        <v>0.37076106043634494</v>
+        <v>0.34746825456114855</v>
       </c>
       <c r="P80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:P$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,P$9))</f>
-        <v>0.41790151635931294</v>
+        <v>0.39635372882237035</v>
       </c>
       <c r="Q80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:Q$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,Q$9))</f>
-        <v>0.47136110874344317</v>
+        <v>0.45179225771102483</v>
       </c>
       <c r="R80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:R$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,R$9))</f>
-        <v>0.52966825809683538</v>
+        <v>0.5122577876502824</v>
       </c>
       <c r="S80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:S$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,S$9))</f>
-        <v>0.59061896696500005</v>
+        <v>0.57546473487299998</v>
       </c>
       <c r="T80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:T$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,T$9))</f>
-        <v>0.65156967583316472</v>
+        <v>0.63867168209571767</v>
       </c>
       <c r="U80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:U$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,U$9))</f>
-        <v>0.70987682518655681</v>
+        <v>0.69913721203497514</v>
       </c>
       <c r="V80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:V$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,V$9))</f>
-        <v>0.76333641757068704</v>
+        <v>0.75457574092362967</v>
       </c>
       <c r="W80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:W$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,W$9))</f>
-        <v>0.81047687349365505</v>
+        <v>0.80346121518485136</v>
       </c>
       <c r="X80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:X$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,X$9))</f>
-        <v>0.85063690122440572</v>
+        <v>0.84510786376987324</v>
       </c>
       <c r="Y80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:Y$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,Y$9))</f>
-        <v>0.88385772902784698</v>
+        <v>0.87955844110784831</v>
       </c>
       <c r="Z80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:Z$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,Z$9))</f>
-        <v>0.91067566127621058</v>
+        <v>0.9073691041784151</v>
       </c>
       <c r="AA80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AA$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AA$9))</f>
-        <v>0.93190135117802309</v>
+        <v>0.92938051448525039</v>
       </c>
       <c r="AB80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AB$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AB$9))</f>
-        <v>0.94843980488741186</v>
+        <v>0.94653117918081209</v>
       </c>
       <c r="AC80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AC$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AC$9))</f>
-        <v>0.96116949409196173</v>
+        <v>0.95973208871336446</v>
       </c>
       <c r="AD80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AD$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AD$9))</f>
-        <v>0.97087565957856936</v>
+        <v>0.96979755146251745</v>
       </c>
       <c r="AE80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AE$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AE$9))</f>
-        <v>0.97822339058775476</v>
+        <v>0.97741727656052824</v>
       </c>
       <c r="AF80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AF$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AF$9))</f>
-        <v>0.98375551028570629</v>
+        <v>0.98315418108996533</v>
       </c>
       <c r="AG80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AG$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AG$9))</f>
-        <v>0.98790358328663208</v>
+        <v>0.98745580507620323</v>
       </c>
       <c r="AH80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AH$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AH$9))</f>
-        <v>0.99100430815198304</v>
+        <v>0.990671310794772</v>
       </c>
       <c r="AI80">
         <f>IF($G80="s-curve",$E80+($F80-$E80)*$O$2/(1+EXP($O$3*(COUNT($I$9:AI$9)+$O$4))),TREND($E80:$F80,$E$9:$F$9,AI$9))</f>
-        <v>0.99331679637819548</v>
-      </c>
-    </row>
-    <row r="81" spans="1:35" x14ac:dyDescent="0.25">
+        <v>0.99306940138275057</v>
+      </c>
+    </row>
+    <row r="81" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C81" t="s">
         <v>38</v>
       </c>
       <c r="D81">
         <f t="shared" si="5"/>
-        <v>1.06995776452E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="E81">
         <f t="shared" si="5"/>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="F81">
         <f t="shared" si="5"/>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="G81" s="5" t="str">
         <f>IF(E81=F81,"n/a",IF(OR(C81="battery electric vehicle",C81="natural gas vehicle",C81="plugin hybrid vehicle"),"s-curve","linear"))</f>
@@ -16103,114 +16205,114 @@
       </c>
       <c r="I81" s="16">
         <f t="shared" si="4"/>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="J81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,J$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="K81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,K$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="L81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,L$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="M81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,M$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="N81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,N$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="O81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,O$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="P81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,P$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Q81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,Q$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="R81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,R$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="S81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,S$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="T81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,T$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="U81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,U$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="V81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,V$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="W81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,W$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="X81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,X$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Y81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,Y$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Z81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,Z$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AA81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AA$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AB81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AB$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AC81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AC$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AD81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AD$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AE81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AE$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AF81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AF$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AG81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AG$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AH81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AH$9))</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AI81">
         <f>IF($G81="s-curve",$E81+($F81-$E81)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E81:$F81,$E$9:$F$9,AI$9))</f>
-        <v>1.06732008758E-4</v>
-      </c>
-    </row>
-    <row r="82" spans="1:35" x14ac:dyDescent="0.25">
+        <v>1.0695408416000001E-4</v>
+      </c>
+    </row>
+    <row r="82" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C82" t="s">
         <v>39</v>
       </c>
@@ -16339,21 +16441,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C83" t="s">
         <v>40</v>
       </c>
       <c r="D83">
         <f t="shared" si="5"/>
-        <v>6.8106756297200005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="E83">
         <f t="shared" si="5"/>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="F83">
         <f t="shared" si="5"/>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="G83" s="5" t="str">
         <f>IF(E83=F83,"n/a",IF(OR(C83="battery electric vehicle",C83="natural gas vehicle",C83="plugin hybrid vehicle"),"s-curve","linear"))</f>
@@ -16361,128 +16463,128 @@
       </c>
       <c r="I83" s="16">
         <f t="shared" si="4"/>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="J83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,J$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="K83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,K$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="L83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,L$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="M83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,M$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="N83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,N$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="O83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,O$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="P83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,P$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Q83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,Q$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="R83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,R$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="S83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,S$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="T83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,T$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="U83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,U$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="V83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,V$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="W83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,W$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="X83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,X$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Y83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,Y$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Z83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,Z$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AA83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AA$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AB83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AB$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AC83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AC$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AD83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AD$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AE83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AE$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AF83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AF$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AG83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AG$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AH83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AH$9))</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AI83">
         <f>IF($G83="s-curve",$E83+($F83-$E83)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E83:$F83,$E$9:$F$9,AI$9))</f>
-        <v>6.7938858436000005E-2</v>
-      </c>
-    </row>
-    <row r="84" spans="1:35" x14ac:dyDescent="0.25">
+        <v>6.7938939010499994E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C84" t="s">
         <v>41</v>
       </c>
       <c r="D84">
         <f t="shared" si="5"/>
-        <v>1.6603971957400002E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="E84">
         <f t="shared" si="5"/>
-        <v>1.3970074369600001E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="F84">
         <f t="shared" si="5"/>
-        <v>9.1136971557240806E-2</v>
+        <v>9.1008967024832244E-2</v>
       </c>
       <c r="G84" s="5" t="str">
         <f>IF(E84=F84,"n/a",IF(OR(C84="battery electric vehicle",C84="natural gas vehicle",C84="plugin hybrid vehicle"),"s-curve","linear"))</f>
@@ -16490,114 +16592,114 @@
       </c>
       <c r="I84" s="16">
         <f t="shared" si="4"/>
-        <v>1.3970074369600001E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="J84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:J$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,J$9))</f>
-        <v>1.5110140554321749E-2</v>
+        <v>1.2806537318706219E-2</v>
       </c>
       <c r="K84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:K$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,K$9))</f>
-        <v>1.550108920235292E-2</v>
+        <v>1.3208673429906077E-2</v>
       </c>
       <c r="L84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:L$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,L$9))</f>
-        <v>1.6022481838446352E-2</v>
+        <v>1.3744986339907847E-2</v>
       </c>
       <c r="M84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:M$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,M$9))</f>
-        <v>1.6714992675043627E-2</v>
+        <v>1.4457314202391682E-2</v>
       </c>
       <c r="N84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:N$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,N$9))</f>
-        <v>1.7629781849127387E-2</v>
+        <v>1.5398281162851517E-2</v>
       </c>
       <c r="O84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:O$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,O$9))</f>
-        <v>1.8829532862010948E-2</v>
+        <v>1.663236448596514E-2</v>
       </c>
       <c r="P84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:P$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,P$9))</f>
-        <v>2.0388253288765361E-2</v>
+        <v>1.8235689562083129E-2</v>
       </c>
       <c r="Q84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:Q$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,Q$9))</f>
-        <v>2.2388737554300295E-2</v>
+        <v>2.0293420077612576E-2</v>
       </c>
       <c r="R84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:R$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,R$9))</f>
-        <v>2.4916280910733307E-2</v>
+        <v>2.2893292110330199E-2</v>
       </c>
       <c r="S84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:S$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,S$9))</f>
-        <v>2.8047286009566623E-2</v>
+        <v>2.611389466499453E-2</v>
       </c>
       <c r="T84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:T$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,T$9))</f>
-        <v>3.18322986028182E-2</v>
+        <v>3.0007219920774212E-2</v>
       </c>
       <c r="U84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:U$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,U$9))</f>
-        <v>3.6275204382572757E-2</v>
+        <v>3.4577264763480553E-2</v>
       </c>
       <c r="V84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:V$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,V$9))</f>
-        <v>4.1313677756162917E-2</v>
+        <v>3.9759920079065703E-2</v>
       </c>
       <c r="W84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:W$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,W$9))</f>
-        <v>4.6809024922225891E-2</v>
+        <v>4.5412523177152192E-2</v>
       </c>
       <c r="X84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:X$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,X$9))</f>
-        <v>5.2553522963420404E-2</v>
+        <v>5.1321406900666118E-2</v>
       </c>
       <c r="Y84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:Y$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,Y$9))</f>
-        <v>5.8298021004614918E-2</v>
+        <v>5.7230290624180044E-2</v>
       </c>
       <c r="Z84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:Z$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,Z$9))</f>
-        <v>6.3793368170677878E-2</v>
+        <v>6.2882893722266534E-2</v>
       </c>
       <c r="AA84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AA$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AA$9))</f>
-        <v>6.8831841544268038E-2</v>
+        <v>6.8065549037851683E-2</v>
       </c>
       <c r="AB84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AB$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AB$9))</f>
-        <v>7.3274747324022602E-2</v>
+        <v>7.2635593880558014E-2</v>
       </c>
       <c r="AC84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AC$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AC$9))</f>
-        <v>7.7059759917274179E-2</v>
+        <v>7.6528919136337692E-2</v>
       </c>
       <c r="AD84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AD$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AD$9))</f>
-        <v>8.0190765016107501E-2</v>
+        <v>7.9749521691002051E-2</v>
       </c>
       <c r="AE84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AE$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AE$9))</f>
-        <v>8.2718308372540517E-2</v>
+        <v>8.234939372371966E-2</v>
       </c>
       <c r="AF84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AF$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AF$9))</f>
-        <v>8.4718792638075455E-2</v>
+        <v>8.4407124239249121E-2</v>
       </c>
       <c r="AG84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AG$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AG$9))</f>
-        <v>8.6277513064829864E-2</v>
+        <v>8.601044931536711E-2</v>
       </c>
       <c r="AH84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AH$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AH$9))</f>
-        <v>8.7477264077713432E-2</v>
+        <v>8.7244532638480726E-2</v>
       </c>
       <c r="AI84">
         <f>IF($G84="s-curve",$E84+($F84-$E84)*$I$2/(1+EXP($I$3*(COUNT($I$9:AI$9)+$I$4))),TREND($E84:$F84,$E$9:$F$9,AI$9))</f>
-        <v>8.8392053251797179E-2</v>
-      </c>
-    </row>
-    <row r="85" spans="1:35" x14ac:dyDescent="0.25">
+        <v>8.8185499598940564E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C85" t="s">
         <v>42</v>
       </c>
@@ -16726,7 +16828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A86" s="17"/>
       <c r="B86" s="17"/>
       <c r="C86" s="17" t="s">
@@ -16857,7 +16959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>49</v>
       </c>
@@ -16986,7 +17088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C88" t="s">
         <v>38</v>
       </c>
@@ -17109,7 +17211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C89" t="s">
         <v>39</v>
       </c>
@@ -17232,7 +17334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C90" t="s">
         <v>40</v>
       </c>
@@ -17355,7 +17457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C91" t="s">
         <v>41</v>
       </c>
@@ -17478,7 +17580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:35" x14ac:dyDescent="0.3">
       <c r="C92" t="s">
         <v>42</v>
       </c>
@@ -17601,7 +17703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A93" s="17"/>
       <c r="B93" s="17"/>
       <c r="C93" s="17" t="s">
@@ -17742,13 +17844,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -17861,233 +17963,233 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
       <c r="B2">
         <f>Data!I10</f>
-        <v>0.18218700570900001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="C2">
         <f>Data!J10</f>
-        <v>0.18123793393000001</v>
+        <v>0.15092946974599999</v>
       </c>
       <c r="D2">
         <f>Data!K10</f>
-        <v>0.22006843983803839</v>
+        <v>0.19119738103263559</v>
       </c>
       <c r="E2">
         <f>Data!L10</f>
-        <v>0.23279812904258823</v>
+        <v>0.20439829056518796</v>
       </c>
       <c r="F2">
         <f>Data!M10</f>
-        <v>0.24933658275197695</v>
+        <v>0.22154895526074969</v>
       </c>
       <c r="G2">
         <f>Data!N10</f>
-        <v>0.2705622726537894</v>
+        <v>0.24356036556758487</v>
       </c>
       <c r="H2">
         <f>Data!O10</f>
-        <v>0.29738020490215311</v>
+        <v>0.27137102863815177</v>
       </c>
       <c r="I2">
         <f>Data!P10</f>
-        <v>0.33060103270559432</v>
+        <v>0.30582160597612668</v>
       </c>
       <c r="J2">
         <f>Data!Q10</f>
-        <v>0.37076106043634494</v>
+        <v>0.34746825456114855</v>
       </c>
       <c r="K2">
         <f>Data!R10</f>
-        <v>0.41790151635931294</v>
+        <v>0.39635372882237035</v>
       </c>
       <c r="L2">
         <f>Data!S10</f>
-        <v>0.47136110874344317</v>
+        <v>0.45179225771102483</v>
       </c>
       <c r="M2">
         <f>Data!T10</f>
-        <v>0.52966825809683538</v>
+        <v>0.5122577876502824</v>
       </c>
       <c r="N2">
         <f>Data!U10</f>
-        <v>0.59061896696500005</v>
+        <v>0.57546473487299998</v>
       </c>
       <c r="O2">
         <f>Data!V10</f>
-        <v>0.65156967583316472</v>
+        <v>0.63867168209571767</v>
       </c>
       <c r="P2">
         <f>Data!W10</f>
-        <v>0.70987682518655681</v>
+        <v>0.69913721203497514</v>
       </c>
       <c r="Q2">
         <f>Data!X10</f>
-        <v>0.76333641757068704</v>
+        <v>0.75457574092362967</v>
       </c>
       <c r="R2">
         <f>Data!Y10</f>
-        <v>0.81047687349365505</v>
+        <v>0.80346121518485136</v>
       </c>
       <c r="S2">
         <f>Data!Z10</f>
-        <v>0.85063690122440572</v>
+        <v>0.84510786376987324</v>
       </c>
       <c r="T2">
         <f>Data!AA10</f>
-        <v>0.88385772902784698</v>
+        <v>0.87955844110784831</v>
       </c>
       <c r="U2">
         <f>Data!AB10</f>
-        <v>0.91067566127621058</v>
+        <v>0.9073691041784151</v>
       </c>
       <c r="V2">
         <f>Data!AC10</f>
-        <v>0.93190135117802309</v>
+        <v>0.92938051448525039</v>
       </c>
       <c r="W2">
         <f>Data!AD10</f>
-        <v>0.94843980488741186</v>
+        <v>0.94653117918081209</v>
       </c>
       <c r="X2">
         <f>Data!AE10</f>
-        <v>0.96116949409196173</v>
+        <v>0.95973208871336446</v>
       </c>
       <c r="Y2">
         <f>Data!AF10</f>
-        <v>0.97087565957856936</v>
+        <v>0.96979755146251745</v>
       </c>
       <c r="Z2">
         <f>Data!AG10</f>
-        <v>0.97822339058775476</v>
+        <v>0.97741727656052824</v>
       </c>
       <c r="AA2">
         <f>Data!AH10</f>
-        <v>0.98375551028570629</v>
+        <v>0.98315418108996533</v>
       </c>
       <c r="AB2">
         <f>Data!AI10</f>
-        <v>0.98790358328663208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+        <v>0.98745580507620323</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
       <c r="B3">
         <f>Data!I11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="C3">
         <f>Data!J11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="D3">
         <f>Data!K11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="E3">
         <f>Data!L11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="F3">
         <f>Data!M11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="G3">
         <f>Data!N11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="H3">
         <f>Data!O11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="I3">
         <f>Data!P11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="J3">
         <f>Data!Q11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="K3">
         <f>Data!R11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="L3">
         <f>Data!S11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="M3">
         <f>Data!T11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="N3">
         <f>Data!U11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="O3">
         <f>Data!V11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="P3">
         <f>Data!W11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Q3">
         <f>Data!X11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="R3">
         <f>Data!Y11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="S3">
         <f>Data!Z11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="T3">
         <f>Data!AA11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="U3">
         <f>Data!AB11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="V3">
         <f>Data!AC11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="W3">
         <f>Data!AD11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="X3">
         <f>Data!AE11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Y3">
         <f>Data!AF11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="Z3">
         <f>Data!AG11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AA3">
         <f>Data!AH11</f>
-        <v>1.06732008758E-4</v>
+        <v>1.0695408416000001E-4</v>
       </c>
       <c r="AB3">
         <f>Data!AI11</f>
-        <v>1.06732008758E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+        <v>1.0695408416000001E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -18200,233 +18302,233 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
       <c r="B5">
         <f>Data!I13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="C5">
         <f>Data!J13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="D5">
         <f>Data!K13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="E5">
         <f>Data!L13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="F5">
         <f>Data!M13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="G5">
         <f>Data!N13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="H5">
         <f>Data!O13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="I5">
         <f>Data!P13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="J5">
         <f>Data!Q13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="K5">
         <f>Data!R13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="L5">
         <f>Data!S13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="M5">
         <f>Data!T13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="N5">
         <f>Data!U13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="O5">
         <f>Data!V13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="P5">
         <f>Data!W13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Q5">
         <f>Data!X13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="R5">
         <f>Data!Y13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="S5">
         <f>Data!Z13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="T5">
         <f>Data!AA13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="U5">
         <f>Data!AB13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="V5">
         <f>Data!AC13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="W5">
         <f>Data!AD13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="X5">
         <f>Data!AE13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Y5">
         <f>Data!AF13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="Z5">
         <f>Data!AG13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AA5">
         <f>Data!AH13</f>
-        <v>6.7938858436000005E-2</v>
+        <v>6.7938939010499994E-2</v>
       </c>
       <c r="AB5">
         <f>Data!AI13</f>
-        <v>6.7938858436000005E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+        <v>6.7938939010499994E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
       <c r="B6">
         <f>Data!I14</f>
-        <v>1.6603971957400002E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="C6">
         <f>Data!J14</f>
-        <v>1.3970074369600001E-2</v>
+        <v>1.1633846776499999E-2</v>
       </c>
       <c r="D6">
         <f>Data!K14</f>
-        <v>1.6992371673937554E-2</v>
+        <v>1.4742630733106016E-2</v>
       </c>
       <c r="E6">
         <f>Data!L14</f>
-        <v>1.8393603157554242E-2</v>
+        <v>1.6183960131609255E-2</v>
       </c>
       <c r="F6">
         <f>Data!M14</f>
-        <v>2.0388253288765361E-2</v>
+        <v>1.8235689562083126E-2</v>
       </c>
       <c r="G6">
         <f>Data!N14</f>
-        <v>2.3168593997747108E-2</v>
+        <v>2.109559304595815E-2</v>
       </c>
       <c r="H6">
         <f>Data!O14</f>
-        <v>2.6932694373384324E-2</v>
+        <v>2.4967407656003776E-2</v>
       </c>
       <c r="I6">
         <f>Data!P14</f>
-        <v>3.18322986028182E-2</v>
+        <v>3.0007219920774209E-2</v>
       </c>
       <c r="J6">
         <f>Data!Q14</f>
-        <v>3.7893781709970521E-2</v>
+        <v>3.6242159617047354E-2</v>
       </c>
       <c r="K6">
         <f>Data!R14</f>
-        <v>4.493810244183398E-2</v>
+        <v>4.3488062012213696E-2</v>
       </c>
       <c r="L6">
         <f>Data!S14</f>
-        <v>5.2553522963420404E-2</v>
+        <v>5.1321406900666118E-2</v>
       </c>
       <c r="M6">
         <f>Data!T14</f>
-        <v>6.0168943485006829E-2</v>
+        <v>5.9154751789118533E-2</v>
       </c>
       <c r="N6">
         <f>Data!U14</f>
-        <v>6.721326421687028E-2</v>
+        <v>6.6400654184284882E-2</v>
       </c>
       <c r="O6">
         <f>Data!V14</f>
-        <v>7.3274747324022602E-2</v>
+        <v>7.2635593880558028E-2</v>
       </c>
       <c r="P6">
         <f>Data!W14</f>
-        <v>7.8174351553456478E-2</v>
+        <v>7.7675406145328446E-2</v>
       </c>
       <c r="Q6">
         <f>Data!X14</f>
-        <v>8.1938451929093686E-2</v>
+        <v>8.1547220755374072E-2</v>
       </c>
       <c r="R6">
         <f>Data!Y14</f>
-        <v>8.4718792638075455E-2</v>
+        <v>8.4407124239249121E-2</v>
       </c>
       <c r="S6">
         <f>Data!Z14</f>
-        <v>8.6713442769286567E-2</v>
+        <v>8.6458853669722974E-2</v>
       </c>
       <c r="T6">
         <f>Data!AA14</f>
-        <v>8.8114674252903258E-2</v>
+        <v>8.7900183068226223E-2</v>
       </c>
       <c r="U6">
         <f>Data!AB14</f>
-        <v>8.908456408839445E-2</v>
+        <v>8.8897827461424384E-2</v>
       </c>
       <c r="V6">
         <f>Data!AC14</f>
-        <v>8.9749031542300767E-2</v>
+        <v>8.9581309446279456E-2</v>
       </c>
       <c r="W6">
         <f>Data!AD14</f>
-        <v>9.0201057861762329E-2</v>
+        <v>9.0046271039531389E-2</v>
       </c>
       <c r="X6">
         <f>Data!AE14</f>
-        <v>9.050709126827812E-2</v>
+        <v>9.0361061958014605E-2</v>
       </c>
       <c r="Y6">
         <f>Data!AF14</f>
-        <v>9.0713610894126245E-2</v>
+        <v>9.0573491389970062E-2</v>
       </c>
       <c r="Z6">
         <f>Data!AG14</f>
-        <v>9.0852670195706434E-2</v>
+        <v>9.0716530039790799E-2</v>
       </c>
       <c r="AA6">
         <f>Data!AH14</f>
-        <v>9.0946166900329001E-2</v>
+        <v>9.0812702264445544E-2</v>
       </c>
       <c r="AB6">
         <f>Data!AI14</f>
-        <v>9.1008967024832244E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+        <v>9.0877299489625335E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -18539,7 +18641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -18663,12 +18765,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -18781,7 +18883,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -18791,7 +18893,7 @@
       </c>
       <c r="C2">
         <f>Data!J17</f>
-        <v>0.30713450135322462</v>
+        <v>0.30732944248799998</v>
       </c>
       <c r="D2">
         <f>Data!K17</f>
@@ -18894,7 +18996,7 @@
         <v>0.30014541837982223</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -19007,7 +19109,7 @@
         <v>0.59353215226599998</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -19120,7 +19222,7 @@
         <v>0.97401567340499995</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -19233,7 +19335,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -19247,106 +19349,106 @@
       </c>
       <c r="D6">
         <f>Data!K21</f>
-        <v>1.0321237741728829E-3</v>
+        <v>1.0321411607416443E-3</v>
       </c>
       <c r="E6">
         <f>Data!L21</f>
-        <v>1.0318317242370562E-3</v>
+        <v>1.0318549051658338E-3</v>
       </c>
       <c r="F6">
         <f>Data!M21</f>
-        <v>1.0314486991464152E-3</v>
+        <v>1.031479479410095E-3</v>
       </c>
       <c r="G6">
         <f>Data!N21</f>
-        <v>1.0309510717001113E-3</v>
+        <v>1.0309917250444676E-3</v>
       </c>
       <c r="H6">
         <f>Data!O21</f>
-        <v>1.0303124094619435E-3</v>
+        <v>1.030365734060366E-3</v>
       </c>
       <c r="I6">
         <f>Data!P21</f>
-        <v>1.0295054815970778E-3</v>
+        <v>1.0295748158910443E-3</v>
       </c>
       <c r="J6">
         <f>Data!Q21</f>
-        <v>1.028505896267372E-3</v>
+        <v>1.0285950626398874E-3</v>
       </c>
       <c r="K6">
         <f>Data!R21</f>
-        <v>1.0272975165485478E-3</v>
+        <v>1.0274106575441273E-3</v>
       </c>
       <c r="L6">
         <f>Data!S21</f>
-        <v>1.025879101918574E-3</v>
+        <v>1.0260203846940701E-3</v>
       </c>
       <c r="M6">
         <f>Data!T21</f>
-        <v>1.024270550060824E-3</v>
+        <v>1.0244437469969668E-3</v>
       </c>
       <c r="N6">
         <f>Data!U21</f>
-        <v>1.0225161395008146E-3</v>
+        <v>1.0227241444788512E-3</v>
       </c>
       <c r="O6">
         <f>Data!V21</f>
-        <v>1.0206821865728424E-3</v>
+        <v>1.0209265777376718E-3</v>
       </c>
       <c r="P6">
         <f>Data!W21</f>
-        <v>1.0188482336448703E-3</v>
+        <v>1.0191290109964925E-3</v>
       </c>
       <c r="Q6">
         <f>Data!X21</f>
-        <v>1.0170938230848608E-3</v>
+        <v>1.0174094084783769E-3</v>
       </c>
       <c r="R6">
         <f>Data!Y21</f>
-        <v>1.0154852712271109E-3</v>
+        <v>1.0158327707812736E-3</v>
       </c>
       <c r="S6">
         <f>Data!Z21</f>
-        <v>1.0140668565971371E-3</v>
+        <v>1.0144424979312164E-3</v>
       </c>
       <c r="T6">
         <f>Data!AA21</f>
-        <v>1.0128584768783128E-3</v>
+        <v>1.0132580928354563E-3</v>
       </c>
       <c r="U6">
         <f>Data!AB21</f>
-        <v>1.0118588915486071E-3</v>
+        <v>1.0122783395842994E-3</v>
       </c>
       <c r="V6">
         <f>Data!AC21</f>
-        <v>1.0110519636837413E-3</v>
+        <v>1.0114874214149777E-3</v>
       </c>
       <c r="W6">
         <f>Data!AD21</f>
-        <v>1.0104133014455735E-3</v>
+        <v>1.0108614304308761E-3</v>
       </c>
       <c r="X6">
         <f>Data!AE21</f>
-        <v>1.0099156739992697E-3</v>
+        <v>1.0103736760652487E-3</v>
       </c>
       <c r="Y6">
         <f>Data!AF21</f>
-        <v>1.0095326489086287E-3</v>
+        <v>1.0099982503095099E-3</v>
       </c>
       <c r="Z6">
         <f>Data!AG21</f>
-        <v>1.0092405989728019E-3</v>
+        <v>1.0097119947336994E-3</v>
       </c>
       <c r="AA6">
         <f>Data!AH21</f>
-        <v>1.0090195122447148E-3</v>
+        <v>1.0094952944338913E-3</v>
       </c>
       <c r="AB6">
         <f>Data!AI21</f>
-        <v>1.0088530556553437E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+        <v>1.0093321403941448E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -19459,7 +19561,7 @@
         <v>1.3472785756799999E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -19583,12 +19685,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -19701,7 +19803,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -19814,7 +19916,7 @@
         <v>0.73751575888521737</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -19927,7 +20029,7 @@
         <v>1.5317430015500001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -20040,7 +20142,7 @@
         <v>0.38138758163300002</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -20153,7 +20255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -20266,7 +20368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -20379,7 +20481,7 @@
         <v>5.5226931821800003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -20503,12 +20605,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -20621,7 +20723,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -20734,7 +20836,7 @@
         <v>0.24513810124032956</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -20847,7 +20949,7 @@
         <v>2.32516282526E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -20960,7 +21062,7 @@
         <v>7.3518745439599999E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -21073,7 +21175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -21186,7 +21288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -21299,7 +21401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -21423,12 +21525,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -21541,7 +21643,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -21654,7 +21756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -21767,7 +21869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -21880,7 +21982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -21993,7 +22095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -22106,7 +22208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -22219,7 +22321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -22343,12 +22445,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>75</v>
       </c>
@@ -22461,7 +22563,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
@@ -22574,7 +22676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -22687,7 +22789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -22800,7 +22902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -22913,7 +23015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -23026,7 +23128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
@@ -23139,7 +23241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>

</xml_diff>